<commit_message>
refactor(schedule): keep the table named schedule and type import rows
- The entries table is `schedule` (a collective noun, like `feedback`) rather
  than `schedule_entries`; the unmerged migration is edited in place.
- The import spreadsheet gains a `type` column (blank/`event`, or `block`) and
  drops `block_title`: a block row's `title` names the block. Unknown types
  are rejected with INVALID_TYPE; an old-layout file fails on the missing
  `type` column. Template, format guide and error copy updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MuMVu2V9H1cAky5kdM1Xx7
</commit_message>
<xml_diff>
--- a/frontend/static/schedule-template.xlsx
+++ b/frontend/static/schedule-template.xlsx
@@ -14,7 +14,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+  <si>
+    <t>type</t>
+  </si>
   <si>
     <t>number</t>
   </si>
@@ -28,10 +31,10 @@
     <t>nomination_title</t>
   </si>
   <si>
-    <t>block_title</t>
-  </si>
-  <si>
     <t>Открытие фестиваля</t>
+  </si>
+  <si>
+    <t>block</t>
   </si>
   <si>
     <t>Косплей</t>
@@ -430,11 +433,11 @@
   <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" customWidth="1"/>
-    <col min="2" max="2" width="38.7109375" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" customWidth="1"/>
-    <col min="4" max="4" width="26.7109375" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="38.7109375" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -455,83 +458,92 @@
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2">
+      <c r="D2" s="2">
         <v>900</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="E3" t="s">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="B4" s="2">
         <v>1</v>
       </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="2">
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="2">
         <v>45</v>
       </c>
-      <c r="D4" t="s">
-        <v>8</v>
+      <c r="E4" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="B5" s="2">
         <v>2</v>
       </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="2">
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="2">
         <v>480</v>
       </c>
-      <c r="D5" t="s">
-        <v>10</v>
+      <c r="E5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="2">
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="2">
         <v>600</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="E7" t="s">
-        <v>12</v>
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="B8" s="2">
         <v>3</v>
       </c>
-      <c r="B8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="2">
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="2">
         <v>210</v>
       </c>
-      <c r="D8" t="s">
-        <v>14</v>
+      <c r="E8" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="E9" t="s">
-        <v>15</v>
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="B10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="2">
+      <c r="C10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="2">
         <v>1200</v>
       </c>
     </row>

</xml_diff>